<commit_message>
Recalcular balance de materia desde el fermentador de 600 L y unificar el flowsheet
</commit_message>
<xml_diff>
--- a/static/files/planilla-balance-cerveceria-dwsim.xlsx
+++ b/static/files/planilla-balance-cerveceria-dwsim.xlsx
@@ -25,12 +25,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="166">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="260" uniqueCount="179">
   <si>
     <t xml:space="preserve">Planta piloto de cerveza — Balance de materia y energía</t>
   </si>
   <si>
-    <t xml:space="preserve">Insumo y complemento para simular en DWSIM · sin TACC y sin alcohol (≤0,5 % v/v) · lote 650 L</t>
+    <t xml:space="preserve">Insumo y complemento para simular en DWSIM · sin TACC y sin alcohol (≤0,5 % v/v) · fermentador de 600 L</t>
   </si>
   <si>
     <t xml:space="preserve">Cómo usar esta planilla</t>
@@ -45,7 +45,7 @@
     <t xml:space="preserve">• Las celdas en color CREMA con texto azul son las que completás vos (datos de tu receta o resultados que te da DWSIM). El resto son fórmulas — no las edites, se recalculan solas.</t>
   </si>
   <si>
-    <t xml:space="preserve">• Si cambiás el tamaño del lote (celda B6 de la pestaña Balance de materia), todo lo que depende de ese factor de escala se recalcula automáticamente en esa pestaña.</t>
+    <t xml:space="preserve">• El balance de materia se calcula hacia atrás a partir del volumen del fermentador (celda B6 de la pestaña Balance de materia, 600 L por defecto): cambiá ese único dato y toda la planilla se recalcula sola, sin perder la coherencia entre las corrientes.</t>
   </si>
   <si>
     <t xml:space="preserve">Referencia de colores</t>
@@ -102,52 +102,64 @@
     <t xml:space="preserve">Balance de materia del proceso</t>
   </si>
   <si>
-    <t xml:space="preserve">Escalado del lote, reparto de azúcares y cierre entradas = salidas</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escala del lote</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Volumen de lote objetivo (L)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Volumen base de referencia (L)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Factor de escala f = lote / base</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Malta (sin TACC) y azúcares fermentables</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Concepto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Base 20 L (kg)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Escalado (kg)</t>
+    <t xml:space="preserve">Calculado hacia atrás desde el volumen del fermentador — cierra por construcción</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Punto de partida: el fermentador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Variable</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Valor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Unidad</t>
   </si>
   <si>
     <t xml:space="preserve">Nota</t>
   </si>
   <si>
-    <t xml:space="preserve">Malta total</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sorgo, mijo, quinoa u otra semilla sin gluten</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% almidón extraíble (del total de malta)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% maltosa (del almidón)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% glucosa (del almidón) = 1 − % maltosa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Almidón total (= extracto fermentable)</t>
+    <t xml:space="preserve">Volumen del fermentador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El dato de equipo que fija todo el balance — pensado para el resto de la planta y el cálculo de costos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Concentración de azúcar en el mosto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mosto de fuerza moderada, se va a fermentar poco de todas formas</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ρ mosto (densidad)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg/L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Azúcar total = Vol × conc. × ρ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Split maltosa / glucosa (hidrólisis del almidón)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% maltosa (del azúcar total)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Córdova, ESPOCH (2021)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% glucosa = 1 − % maltosa</t>
   </si>
   <si>
     <t xml:space="preserve">Maltosa</t>
@@ -162,27 +174,66 @@
     <t xml:space="preserve">Va al campo 'Glucose' del reactor en DWSIM</t>
   </si>
   <si>
-    <t xml:space="preserve">Malta no convertida (proteínas, cáscara, dextrinas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">No es azúcar fermentable — sale con el bagazo o queda en la cerveza</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Entradas conocidas (escaladas con el mismo factor f)</t>
+    <t xml:space="preserve">Malta y agua de maceración</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% almidón extraíble (de la malta)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">El resto — proteínas, cáscara, dextrinas — no fermenta, sale como bagazo o queda de cuerpo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malta necesaria = azúcar total / % almidón</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Relación agua / malta</t>
+  </si>
+  <si>
+    <t xml:space="preserve">L/kg</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua de macerado = malta × relación</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua de relleno antes del hervor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% de agua que se evapora en el hervor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua final en el mosto frío (= Vol·ρ − azúcares)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua total antes del hervor = agua final / (1 − % evap.)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua de hervido (relleno) = agua total − agua macerado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Entradas conocidas</t>
   </si>
   <si>
     <t xml:space="preserve">Corriente</t>
   </si>
   <si>
-    <t xml:space="preserve">Malta</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Agua (maceración)</t>
+    <t xml:space="preserve">Cantidad (kg)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Malta (sin TACC)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua de macerado</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Agua de hervido (relleno)</t>
   </si>
   <si>
     <t xml:space="preserve">Enzimas</t>
   </si>
   <si>
+    <t xml:space="preserve">≈0,10 kg — completá con tu receta si tenés un dato más preciso</t>
+  </si>
+  <si>
     <t xml:space="preserve">Levadura + agua de inóculo</t>
   </si>
   <si>
@@ -243,15 +294,6 @@
     <t xml:space="preserve">Datos de la corriente y de la bomba</t>
   </si>
   <si>
-    <t xml:space="preserve">Variable</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Valor</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Unidad</t>
-  </si>
-  <si>
     <t xml:space="preserve">ΔP (aumento de presión)</t>
   </si>
   <si>
@@ -261,9 +303,6 @@
     <t xml:space="preserve">η (eficiencia de la bomba)</t>
   </si>
   <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
     <t xml:space="preserve">ρ (densidad del líquido)</t>
   </si>
   <si>
@@ -363,13 +402,13 @@
     <t xml:space="preserve">ṁ (caudal del mosto)</t>
   </si>
   <si>
-    <t xml:space="preserve">kg</t>
+    <t xml:space="preserve">Mosto-4 de la guía: 600,0 kg para un fermentador de 600 L</t>
   </si>
   <si>
     <t xml:space="preserve">Cₚ (calor específico del mosto)</t>
   </si>
   <si>
-    <t xml:space="preserve">El mosto es &gt;90% agua</t>
+    <t xml:space="preserve">El mosto es ~90% agua</t>
   </si>
   <si>
     <t xml:space="preserve">T₁ (temperatura de entrada)</t>
@@ -420,16 +459,19 @@
     <t xml:space="preserve">Glucosa en el mosto</t>
   </si>
   <si>
-    <t xml:space="preserve">Podés traerlo de la pestaña 'Balance de materia'</t>
+    <t xml:space="preserve">Traído de la pestaña 'Balance de materia' (Glucosa)</t>
   </si>
   <si>
     <t xml:space="preserve">Maltosa en el mosto</t>
   </si>
   <si>
+    <t xml:space="preserve">Traído de la pestaña 'Balance de materia' (Maltosa)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Volumen del mosto</t>
   </si>
   <si>
-    <t xml:space="preserve">L</t>
+    <t xml:space="preserve">El volumen del fermentador (pestaña 'Balance de materia')</t>
   </si>
   <si>
     <t xml:space="preserve">Rendimiento etanol/azúcar (estequiometría)</t>
@@ -442,9 +484,6 @@
   </si>
   <si>
     <t xml:space="preserve">Densidad del etanol</t>
-  </si>
-  <si>
-    <t xml:space="preserve">kg/L</t>
   </si>
   <si>
     <t xml:space="preserve">% v/v de alcohol objetivo</t>
@@ -529,17 +568,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="10">
+  <numFmts count="9">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="General"/>
-    <numFmt numFmtId="166" formatCode="0"/>
-    <numFmt numFmtId="167" formatCode="0.00"/>
-    <numFmt numFmtId="168" formatCode="0.000"/>
-    <numFmt numFmtId="169" formatCode="0.0%"/>
+    <numFmt numFmtId="166" formatCode="0.000"/>
+    <numFmt numFmtId="167" formatCode="0.0%"/>
+    <numFmt numFmtId="168" formatCode="0.00"/>
+    <numFmt numFmtId="169" formatCode="0.00%"/>
     <numFmt numFmtId="170" formatCode="0.0000"/>
-    <numFmt numFmtId="171" formatCode="0.0000000"/>
-    <numFmt numFmtId="172" formatCode="0.00%"/>
-    <numFmt numFmtId="173" formatCode="0.0"/>
+    <numFmt numFmtId="171" formatCode="0.0"/>
+    <numFmt numFmtId="172" formatCode="0"/>
   </numFmts>
   <fonts count="12">
     <font>
@@ -749,95 +787,95 @@
       <alignment horizontal="left" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="166" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="171" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="167" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="11" fillId="5" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="169" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="168" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="171" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="170" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="173" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="166" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="169" fontId="10" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="172" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1303,10 +1341,10 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D45"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="16"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="42"/>
   </cols>
@@ -1336,86 +1374,109 @@
       <c r="D4" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="5" t="s">
+      <c r="A6" s="10" t="s">
         <v>27</v>
       </c>
-      <c r="B6" s="10" t="n">
-        <v>650</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="B8" s="14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="5" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="11" t="n">
+        <v>1</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B10" s="15" t="n">
+        <f aca="false">B7*B8*B9</f>
+        <v>60</v>
+      </c>
+      <c r="C10" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="B12" s="3"/>
+      <c r="C12" s="3"/>
+      <c r="D12" s="3"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B14" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="B7" s="10" t="n">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="5" t="s">
+      <c r="C14" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="B8" s="11" t="n">
-        <f aca="false">B6/B7</f>
-        <v>32.5</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A10" s="3" t="s">
+      <c r="D14" s="10" t="s">
         <v>30</v>
-      </c>
-      <c r="B10" s="3"/>
-      <c r="C10" s="3"/>
-      <c r="D10" s="3"/>
-    </row>
-    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A12" s="12" t="s">
-        <v>31</v>
-      </c>
-      <c r="B12" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C12" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D12" s="12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A13" s="5" t="s">
-        <v>35</v>
-      </c>
-      <c r="B13" s="13" t="n">
-        <v>5</v>
-      </c>
-      <c r="C13" s="14" t="n">
-        <f aca="false">B13*B8</f>
-        <v>162.5</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="5" t="s">
-        <v>37</v>
-      </c>
-      <c r="B14" s="16" t="n">
-        <v>0.58</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="B15" s="16" t="n">
+        <v>42</v>
+      </c>
+      <c r="B15" s="14" t="n">
         <v>0.83</v>
+      </c>
+      <c r="C15" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="13" t="s">
+        <v>43</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>39</v>
+        <v>44</v>
       </c>
       <c r="B16" s="17" t="n">
         <f aca="false">1-B15</f>
@@ -1424,274 +1485,388 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
+        <v>45</v>
+      </c>
+      <c r="B17" s="15" t="n">
+        <f aca="false">B10*B15</f>
+        <v>49.8</v>
+      </c>
+      <c r="C17" s="16" t="s">
         <v>40</v>
       </c>
-      <c r="C17" s="14" t="n">
-        <f aca="false">C13*B14</f>
-        <v>94.25</v>
+      <c r="D17" s="13" t="s">
+        <v>46</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>41</v>
-      </c>
-      <c r="C18" s="18" t="n">
-        <f aca="false">C17*B15</f>
-        <v>78.2275</v>
-      </c>
-      <c r="D18" s="15" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A19" s="5" t="s">
-        <v>43</v>
-      </c>
-      <c r="C19" s="18" t="n">
-        <f aca="false">C17*B16</f>
-        <v>16.0225</v>
-      </c>
-      <c r="D19" s="15" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>45</v>
-      </c>
-      <c r="C20" s="14" t="n">
-        <f aca="false">C13-C17</f>
-        <v>68.25</v>
-      </c>
-      <c r="D20" s="15" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A22" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
+      <c r="B18" s="15" t="n">
+        <f aca="false">B10*B16</f>
+        <v>10.2</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D18" s="13" t="s">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A20" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="D20" s="3"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B22" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C22" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D22" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="B23" s="14" t="n">
+        <v>0.58</v>
+      </c>
+      <c r="C23" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="D23" s="13" t="s">
+        <v>51</v>
+      </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B24" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="C24" s="12" t="s">
-        <v>33</v>
-      </c>
-      <c r="D24" s="12" t="s">
-        <v>34</v>
+      <c r="A24" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="B24" s="15" t="n">
+        <f aca="false">B10/B23</f>
+        <v>103.448275862069</v>
+      </c>
+      <c r="C24" s="16" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="B25" s="14" t="n">
-        <f aca="false">B13</f>
-        <v>5</v>
-      </c>
-      <c r="C25" s="14" t="n">
-        <f aca="false">C13</f>
-        <v>162.5</v>
+        <v>53</v>
+      </c>
+      <c r="B25" s="11" t="n">
+        <v>3</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>54</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>50</v>
-      </c>
-      <c r="B26" s="19" t="n">
-        <v>14.6154</v>
-      </c>
-      <c r="C26" s="14" t="n">
-        <f aca="false">B26*B8</f>
-        <v>475.0005</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="B27" s="20" t="n">
-        <v>0.0050154</v>
-      </c>
-      <c r="C27" s="21" t="n">
-        <f aca="false">B27*B8</f>
-        <v>0.1630005</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="5" t="s">
-        <v>52</v>
-      </c>
-      <c r="B28" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C28" s="14" t="n">
-        <f aca="false">B28*B8</f>
-        <v>0</v>
-      </c>
-      <c r="D28" s="15" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="B29" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C29" s="14" t="n">
-        <f aca="false">B29*B8</f>
-        <v>0</v>
-      </c>
-      <c r="D29" s="15" t="s">
-        <v>53</v>
-      </c>
+        <v>55</v>
+      </c>
+      <c r="B26" s="15" t="n">
+        <f aca="false">B24*B25</f>
+        <v>310.344827586207</v>
+      </c>
+      <c r="C26" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="B28" s="3"/>
+      <c r="C28" s="3"/>
+      <c r="D28" s="3"/>
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="B30" s="13" t="n">
-        <v>0</v>
-      </c>
-      <c r="C30" s="14" t="n">
-        <f aca="false">B30*B8</f>
-        <v>0</v>
-      </c>
-      <c r="D30" s="15" t="s">
-        <v>53</v>
+      <c r="A30" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B30" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C30" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D30" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="9" t="s">
-        <v>56</v>
-      </c>
-      <c r="C31" s="18" t="n">
-        <f aca="false">SUM(C25:C30)</f>
-        <v>637.6635005</v>
-      </c>
-    </row>
-    <row r="33" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A33" s="3" t="s">
+      <c r="A31" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="12" t="s">
-        <v>48</v>
-      </c>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12" t="s">
+      <c r="B31" s="14" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C31" s="12" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="D35" s="12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
+      <c r="B32" s="18" t="n">
+        <f aca="false">B7*B9-B10</f>
+        <v>540</v>
+      </c>
+      <c r="C32" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
         <v>59</v>
       </c>
-      <c r="C36" s="13" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="5" t="s">
+      <c r="B33" s="18" t="n">
+        <f aca="false">B32/(1-B31)</f>
+        <v>600</v>
+      </c>
+      <c r="C33" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="C37" s="13" t="n">
-        <v>0</v>
-      </c>
+      <c r="B34" s="15" t="n">
+        <f aca="false">B33-B26</f>
+        <v>289.655172413793</v>
+      </c>
+      <c r="C34" s="16" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A36" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="B36" s="3"/>
+      <c r="C36" s="3"/>
+      <c r="D36" s="3"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="5" t="s">
-        <v>61</v>
-      </c>
-      <c r="C38" s="13" t="n">
-        <v>0</v>
+      <c r="A38" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B38" s="10" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="10"/>
+      <c r="D38" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="5" t="s">
-        <v>62</v>
-      </c>
-      <c r="C39" s="13" t="n">
-        <v>0</v>
+        <v>64</v>
+      </c>
+      <c r="B39" s="18" t="n">
+        <f aca="false">B24</f>
+        <v>103.448275862069</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C40" s="13" t="n">
-        <v>0</v>
+        <v>65</v>
+      </c>
+      <c r="B40" s="18" t="n">
+        <f aca="false">B26</f>
+        <v>310.344827586207</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="C41" s="13" t="n">
+        <v>66</v>
+      </c>
+      <c r="B41" s="18" t="n">
+        <f aca="false">B34</f>
+        <v>289.655172413793</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>67</v>
+      </c>
+      <c r="B42" s="19" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="D42" s="13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>69</v>
+      </c>
+      <c r="B43" s="11" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="9" t="s">
-        <v>65</v>
-      </c>
-      <c r="C42" s="18" t="n">
-        <f aca="false">SUM(C36:C41)</f>
+      <c r="D43" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="B44" s="11" t="n">
         <v>0</v>
       </c>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="9" t="s">
-        <v>66</v>
-      </c>
-      <c r="C43" s="18" t="n">
-        <f aca="false">C31-C42</f>
-        <v>637.6635005</v>
-      </c>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="9" t="s">
-        <v>67</v>
-      </c>
-      <c r="C44" s="22" t="n">
-        <f aca="false">IFERROR((C31-C42)/C31,"")</f>
+      <c r="D44" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
+        <v>72</v>
+      </c>
+      <c r="B45" s="11" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="9" t="s">
+        <v>73</v>
+      </c>
+      <c r="B46" s="15" t="n">
+        <f aca="false">SUM(B39:B45)</f>
+        <v>703.548275862069</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A48" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="B48" s="3"/>
+      <c r="C48" s="3"/>
+      <c r="D48" s="3"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="10" t="s">
+        <v>62</v>
+      </c>
+      <c r="B50" s="10"/>
+      <c r="C50" s="10" t="s">
+        <v>75</v>
+      </c>
+      <c r="D50" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>76</v>
+      </c>
+      <c r="C51" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
+        <v>77</v>
+      </c>
+      <c r="C52" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="5" t="s">
+        <v>78</v>
+      </c>
+      <c r="C53" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="C54" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="5" t="s">
+        <v>80</v>
+      </c>
+      <c r="C55" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="C56" s="11" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="9" t="s">
+        <v>82</v>
+      </c>
+      <c r="C57" s="15" t="n">
+        <f aca="false">SUM(C51:C56)</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="9" t="s">
+        <v>83</v>
+      </c>
+      <c r="C58" s="15" t="n">
+        <f aca="false">B46-C57</f>
+        <v>703.548275862069</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="9" t="s">
+        <v>84</v>
+      </c>
+      <c r="C59" s="20" t="n">
+        <f aca="false">IFERROR((B46-C57)/B46,"")</f>
         <v>1</v>
       </c>
     </row>
-    <row r="45" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A45" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="B45" s="4"/>
-      <c r="C45" s="4"/>
-      <c r="D45" s="4"/>
+    <row r="60" customFormat="false" ht="22.35" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A60" s="4" t="s">
+        <v>85</v>
+      </c>
+      <c r="B60" s="4"/>
+      <c r="C60" s="4"/>
+      <c r="D60" s="4"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="9">
     <mergeCell ref="A1:D1"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="A4:D4"/>
-    <mergeCell ref="A10:D10"/>
-    <mergeCell ref="A22:D22"/>
-    <mergeCell ref="A33:D33"/>
-    <mergeCell ref="A45:D45"/>
+    <mergeCell ref="A12:D12"/>
+    <mergeCell ref="A20:D20"/>
+    <mergeCell ref="A28:D28"/>
+    <mergeCell ref="A36:D36"/>
+    <mergeCell ref="A48:D48"/>
+    <mergeCell ref="A60:D60"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1718,7 +1893,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>69</v>
+        <v>86</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -1726,7 +1901,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -1734,231 +1909,231 @@
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>71</v>
+        <v>88</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>34</v>
+      <c r="A6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>75</v>
-      </c>
-      <c r="B7" s="13" t="n">
+        <v>89</v>
+      </c>
+      <c r="B7" s="11" t="n">
         <v>100000</v>
       </c>
-      <c r="C7" s="23" t="s">
-        <v>76</v>
+      <c r="C7" s="12" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>77</v>
-      </c>
-      <c r="B8" s="16" t="n">
+        <v>91</v>
+      </c>
+      <c r="B8" s="14" t="n">
         <v>0.72</v>
       </c>
-      <c r="C8" s="23" t="s">
-        <v>78</v>
+      <c r="C8" s="12" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>79</v>
-      </c>
-      <c r="B9" s="13" t="n">
+        <v>92</v>
+      </c>
+      <c r="B9" s="11" t="n">
         <v>998</v>
       </c>
-      <c r="C9" s="23" t="s">
-        <v>80</v>
+      <c r="C9" s="12" t="s">
+        <v>93</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="B10" s="13" t="n">
+        <v>94</v>
+      </c>
+      <c r="B10" s="11" t="n">
         <v>4.186</v>
       </c>
-      <c r="C10" s="23" t="s">
-        <v>82</v>
+      <c r="C10" s="12" t="s">
+        <v>95</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>83</v>
-      </c>
-      <c r="B11" s="13" t="n">
+        <v>96</v>
+      </c>
+      <c r="B11" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>84</v>
+      <c r="C11" s="12" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>85</v>
-      </c>
-      <c r="B12" s="13" t="n">
+        <v>98</v>
+      </c>
+      <c r="B12" s="11" t="n">
         <v>101325</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>76</v>
+      <c r="C12" s="12" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="B13" s="13" t="n">
+        <v>99</v>
+      </c>
+      <c r="B13" s="11" t="n">
         <v>2339</v>
       </c>
-      <c r="C13" s="23" t="s">
-        <v>76</v>
-      </c>
-      <c r="D13" s="15" t="s">
-        <v>87</v>
+      <c r="C13" s="12" t="s">
+        <v>90</v>
+      </c>
+      <c r="D13" s="13" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="B15" s="3"/>
       <c r="C15" s="3"/>
       <c r="D15" s="3"/>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="B17" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C17" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" s="12" t="s">
-        <v>90</v>
+      <c r="A17" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B17" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C17" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D17" s="10" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>91</v>
-      </c>
-      <c r="B18" s="14" t="n">
+        <v>104</v>
+      </c>
+      <c r="B18" s="18" t="n">
         <f aca="false">B7/B9/1000</f>
         <v>0.100200400801603</v>
       </c>
-      <c r="C18" s="24" t="s">
-        <v>92</v>
+      <c r="C18" s="16" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>93</v>
-      </c>
-      <c r="B19" s="14" t="n">
+        <v>106</v>
+      </c>
+      <c r="B19" s="18" t="n">
         <f aca="false">B18/B8</f>
         <v>0.13916722333556</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>92</v>
+      <c r="C19" s="16" t="s">
+        <v>105</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>94</v>
+        <v>107</v>
       </c>
       <c r="B20" s="21" t="n">
         <f aca="false">(B19-B18)/B10</f>
         <v>0.00930884437027158</v>
       </c>
-      <c r="C20" s="24" t="s">
-        <v>95</v>
+      <c r="C20" s="16" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>96</v>
-      </c>
-      <c r="B21" s="25" t="n">
+        <v>109</v>
+      </c>
+      <c r="B21" s="22" t="n">
         <f aca="false">B11*B19</f>
         <v>0.06958361166778</v>
       </c>
-      <c r="C21" s="24" t="s">
-        <v>97</v>
+      <c r="C21" s="16" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="B22" s="14" t="n">
+        <v>111</v>
+      </c>
+      <c r="B22" s="18" t="n">
         <f aca="false">B7/(B9*9.81)</f>
         <v>10.21410813472</v>
       </c>
-      <c r="C22" s="24" t="s">
-        <v>99</v>
+      <c r="C22" s="16" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="B23" s="18" t="n">
+        <v>113</v>
+      </c>
+      <c r="B23" s="15" t="n">
         <f aca="false">(B12-B13)/(B9*9.81)</f>
         <v>10.1105370782339</v>
       </c>
-      <c r="C23" s="24" t="s">
-        <v>99</v>
+      <c r="C23" s="16" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="B25" s="3"/>
       <c r="C25" s="3"/>
       <c r="D25" s="3"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="B27" s="12" t="s">
+      <c r="A27" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="C27" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D27" s="12" t="s">
-        <v>104</v>
+      <c r="B27" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="C27" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D27" s="10" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>105</v>
+        <v>118</v>
       </c>
       <c r="B28" s="21" t="n">
         <f aca="false">B20</f>
         <v>0.00930884437027158</v>
       </c>
-      <c r="C28" s="19" t="n">
+      <c r="C28" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D28" s="17" t="str">
@@ -1968,13 +2143,13 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>106</v>
+        <v>119</v>
       </c>
       <c r="B29" s="21" t="n">
         <f aca="false">B21</f>
         <v>0.06958361166778</v>
       </c>
-      <c r="C29" s="19" t="n">
+      <c r="C29" s="23" t="n">
         <v>0</v>
       </c>
       <c r="D29" s="17" t="str">
@@ -1984,13 +2159,13 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>107</v>
-      </c>
-      <c r="B30" s="14" t="n">
+        <v>120</v>
+      </c>
+      <c r="B30" s="18" t="n">
         <f aca="false">B23</f>
         <v>10.1105370782339</v>
       </c>
-      <c r="C30" s="13" t="n">
+      <c r="C30" s="11" t="n">
         <v>0</v>
       </c>
       <c r="D30" s="17" t="str">
@@ -2031,7 +2206,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>108</v>
+        <v>121</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2039,7 +2214,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>109</v>
+        <v>122</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2047,185 +2222,188 @@
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>110</v>
+        <v>123</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>111</v>
-      </c>
-      <c r="B7" s="13" t="n">
-        <v>700</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>112</v>
+        <v>124</v>
+      </c>
+      <c r="B7" s="11" t="n">
+        <v>600</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>125</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" s="13" t="n">
+        <v>126</v>
+      </c>
+      <c r="B8" s="11" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="23" t="s">
-        <v>82</v>
-      </c>
-      <c r="D8" s="15" t="s">
-        <v>114</v>
+      <c r="C8" s="12" t="s">
+        <v>95</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>115</v>
-      </c>
-      <c r="B9" s="13" t="n">
+        <v>128</v>
+      </c>
+      <c r="B9" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="C9" s="23" t="s">
-        <v>95</v>
+      <c r="C9" s="12" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>116</v>
-      </c>
-      <c r="B10" s="13" t="n">
+        <v>129</v>
+      </c>
+      <c r="B10" s="11" t="n">
         <v>20</v>
       </c>
-      <c r="C10" s="23" t="s">
-        <v>95</v>
+      <c r="C10" s="12" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B11" s="13" t="n">
+        <v>130</v>
+      </c>
+      <c r="B11" s="11" t="n">
         <v>30</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>118</v>
+      <c r="C11" s="12" t="s">
+        <v>131</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>88</v>
+        <v>101</v>
       </c>
       <c r="B13" s="3"/>
       <c r="C13" s="3"/>
       <c r="D13" s="3"/>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="B15" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C15" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D15" s="12" t="s">
-        <v>90</v>
+      <c r="A15" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B15" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C15" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D15" s="10" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="B16" s="26" t="n">
+        <v>132</v>
+      </c>
+      <c r="B16" s="24" t="n">
         <f aca="false">B9-B10</f>
         <v>80</v>
       </c>
-      <c r="C16" s="24" t="s">
-        <v>95</v>
+      <c r="C16" s="16" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B17" s="27" t="n">
+        <v>133</v>
+      </c>
+      <c r="B17" s="25" t="n">
         <f aca="false">B7*B8*B16</f>
-        <v>224000</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>121</v>
+        <v>192000</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="B18" s="28" t="n">
+        <v>135</v>
+      </c>
+      <c r="B18" s="26" t="n">
         <f aca="false">B17/3600</f>
-        <v>62.2222222222222</v>
-      </c>
-      <c r="C18" s="24" t="s">
-        <v>123</v>
+        <v>53.3333333333333</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>124</v>
-      </c>
-      <c r="B19" s="11" t="n">
+        <v>137</v>
+      </c>
+      <c r="B19" s="27" t="n">
         <f aca="false">B17/(B11*60)</f>
-        <v>124.444444444444</v>
-      </c>
-      <c r="C19" s="24" t="s">
-        <v>97</v>
+        <v>106.666666666667</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>110</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A21" s="3" t="s">
-        <v>101</v>
+        <v>114</v>
       </c>
       <c r="B21" s="3"/>
       <c r="C21" s="3"/>
       <c r="D21" s="3"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="B23" s="12" t="s">
+      <c r="A23" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="C23" s="12" t="s">
-        <v>125</v>
-      </c>
-      <c r="D23" s="12" t="s">
-        <v>104</v>
+      <c r="B23" s="10" t="s">
+        <v>115</v>
+      </c>
+      <c r="C23" s="10" t="s">
+        <v>138</v>
+      </c>
+      <c r="D23" s="10" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>126</v>
-      </c>
-      <c r="B24" s="29" t="n">
+        <v>139</v>
+      </c>
+      <c r="B24" s="28" t="n">
         <f aca="false">B17</f>
-        <v>224000</v>
-      </c>
-      <c r="C24" s="10" t="n">
+        <v>192000</v>
+      </c>
+      <c r="C24" s="29" t="n">
         <v>0</v>
       </c>
       <c r="D24" s="17" t="str">
@@ -2266,7 +2444,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>127</v>
+        <v>140</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2274,7 +2452,7 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>128</v>
+        <v>141</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
@@ -2282,239 +2460,248 @@
     </row>
     <row r="4" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>129</v>
+        <v>142</v>
       </c>
       <c r="B4" s="3"/>
       <c r="C4" s="3"/>
       <c r="D4" s="3"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="B6" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C6" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D6" s="12" t="s">
-        <v>34</v>
+      <c r="A6" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B6" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C6" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D6" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>130</v>
-      </c>
-      <c r="B7" s="13" t="n">
-        <v>6.4</v>
-      </c>
-      <c r="C7" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="D7" s="15" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>143</v>
+      </c>
+      <c r="B7" s="18" t="n">
+        <f aca="false">'Balance de materia'!B18</f>
+        <v>10.2</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D7" s="13" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="B8" s="13" t="n">
-        <v>63.2</v>
-      </c>
-      <c r="C8" s="23" t="s">
-        <v>112</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>145</v>
+      </c>
+      <c r="B8" s="18" t="n">
+        <f aca="false">'Balance de materia'!B17</f>
+        <v>49.8</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="B9" s="13" t="n">
-        <v>700</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>134</v>
+        <v>147</v>
+      </c>
+      <c r="B9" s="28" t="n">
+        <f aca="false">'Balance de materia'!B7</f>
+        <v>600</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D9" s="13" t="s">
+        <v>148</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>135</v>
-      </c>
-      <c r="B10" s="13" t="n">
+        <v>149</v>
+      </c>
+      <c r="B10" s="11" t="n">
         <v>0.53</v>
       </c>
-      <c r="C10" s="23" t="s">
-        <v>136</v>
-      </c>
-      <c r="D10" s="15" t="s">
-        <v>137</v>
+      <c r="C10" s="12" t="s">
+        <v>150</v>
+      </c>
+      <c r="D10" s="13" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="B11" s="13" t="n">
+        <v>152</v>
+      </c>
+      <c r="B11" s="11" t="n">
         <v>0.789</v>
       </c>
-      <c r="C11" s="23" t="s">
-        <v>139</v>
+      <c r="C11" s="12" t="s">
+        <v>38</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>140</v>
+        <v>153</v>
       </c>
       <c r="B12" s="30" t="n">
         <v>0.005</v>
       </c>
-      <c r="C12" s="23" t="s">
-        <v>141</v>
-      </c>
-      <c r="D12" s="15" t="s">
-        <v>142</v>
+      <c r="C12" s="12" t="s">
+        <v>154</v>
+      </c>
+      <c r="D12" s="13" t="s">
+        <v>155</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>143</v>
+        <v>156</v>
       </c>
       <c r="B14" s="3"/>
       <c r="C14" s="3"/>
       <c r="D14" s="3"/>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="12" t="s">
-        <v>89</v>
-      </c>
-      <c r="B16" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C16" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D16" s="12" t="s">
-        <v>90</v>
+      <c r="A16" s="10" t="s">
+        <v>102</v>
+      </c>
+      <c r="B16" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C16" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D16" s="10" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>144</v>
-      </c>
-      <c r="B17" s="14" t="n">
+        <v>157</v>
+      </c>
+      <c r="B17" s="18" t="n">
         <f aca="false">B7+B8</f>
-        <v>69.6</v>
-      </c>
-      <c r="C17" s="24" t="s">
-        <v>112</v>
+        <v>60</v>
+      </c>
+      <c r="C17" s="16" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>145</v>
-      </c>
-      <c r="B18" s="14" t="n">
+        <v>158</v>
+      </c>
+      <c r="B18" s="18" t="n">
         <f aca="false">B17*B10</f>
-        <v>36.888</v>
-      </c>
-      <c r="C18" s="24" t="s">
-        <v>112</v>
+        <v>31.8</v>
+      </c>
+      <c r="C18" s="16" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>146</v>
-      </c>
-      <c r="B19" s="28" t="n">
+        <v>159</v>
+      </c>
+      <c r="B19" s="26" t="n">
         <f aca="false">B12*B11*1000</f>
         <v>3.945</v>
       </c>
-      <c r="C19" s="24" t="s">
-        <v>147</v>
+      <c r="C19" s="16" t="s">
+        <v>160</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="B20" s="14" t="n">
+        <v>161</v>
+      </c>
+      <c r="B20" s="18" t="n">
         <f aca="false">B19*B9/1000</f>
-        <v>2.7615</v>
-      </c>
-      <c r="C20" s="24" t="s">
-        <v>112</v>
+        <v>2.367</v>
+      </c>
+      <c r="C20" s="16" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>149</v>
+        <v>162</v>
       </c>
       <c r="B21" s="31" t="n">
         <f aca="false">IFERROR(B20/B18,"")</f>
-        <v>0.0748617436564737</v>
-      </c>
-      <c r="C21" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="D21" s="15" t="s">
-        <v>151</v>
+        <v>0.074433962264151</v>
+      </c>
+      <c r="C21" s="16" t="s">
+        <v>163</v>
+      </c>
+      <c r="D21" s="13" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="18" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A23" s="3" t="s">
-        <v>152</v>
+        <v>165</v>
       </c>
       <c r="B23" s="3"/>
       <c r="C23" s="3"/>
       <c r="D23" s="3"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="12" t="s">
-        <v>72</v>
-      </c>
-      <c r="B25" s="12" t="s">
-        <v>73</v>
-      </c>
-      <c r="C25" s="12" t="s">
-        <v>74</v>
-      </c>
-      <c r="D25" s="12" t="s">
-        <v>34</v>
+      <c r="A25" s="10" t="s">
+        <v>27</v>
+      </c>
+      <c r="B25" s="10" t="s">
+        <v>28</v>
+      </c>
+      <c r="C25" s="10" t="s">
+        <v>29</v>
+      </c>
+      <c r="D25" s="10" t="s">
+        <v>30</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="5" t="s">
-        <v>153</v>
-      </c>
-      <c r="B26" s="16" t="n">
+        <v>166</v>
+      </c>
+      <c r="B26" s="14" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B27" s="13" t="n">
+        <v>167</v>
+      </c>
+      <c r="B27" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="C27" s="24" t="s">
-        <v>112</v>
+      <c r="C27" s="16" t="s">
+        <v>40</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
-        <v>155</v>
-      </c>
-      <c r="B28" s="22" t="str">
+        <v>168</v>
+      </c>
+      <c r="B28" s="20" t="str">
         <f aca="false">IF(B27=0,"",IFERROR((B27/B11)/B9*100,""))</f>
         <v/>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="5" t="s">
-        <v>156</v>
+        <v>169</v>
       </c>
       <c r="B29" s="7" t="str">
         <f aca="false">IF(B28="","",IF(B28&lt;=B12,"Sí","No — bajá el Conversion% y volvé a correr"))</f>
@@ -2554,7 +2741,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>157</v>
+        <v>170</v>
       </c>
       <c r="B1" s="1"/>
       <c r="C1" s="1"/>
@@ -2562,29 +2749,29 @@
     </row>
     <row r="2" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>158</v>
+        <v>171</v>
       </c>
       <c r="B2" s="2"/>
       <c r="C2" s="2"/>
       <c r="D2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="12" t="s">
-        <v>159</v>
-      </c>
-      <c r="B4" s="12" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="12" t="s">
-        <v>103</v>
-      </c>
-      <c r="D4" s="12" t="s">
-        <v>104</v>
+      <c r="A4" s="10" t="s">
+        <v>172</v>
+      </c>
+      <c r="B4" s="10" t="s">
+        <v>101</v>
+      </c>
+      <c r="C4" s="10" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="10" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="5" t="s">
-        <v>160</v>
+        <v>173</v>
       </c>
       <c r="B5" s="21" t="n">
         <f aca="false">Bomba!B20</f>
@@ -2601,7 +2788,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="5" t="s">
-        <v>161</v>
+        <v>174</v>
       </c>
       <c r="B6" s="21" t="n">
         <f aca="false">Bomba!B21</f>
@@ -2618,13 +2805,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="5" t="s">
-        <v>162</v>
-      </c>
-      <c r="B7" s="14" t="n">
+        <v>175</v>
+      </c>
+      <c r="B7" s="18" t="n">
         <f aca="false">Bomba!B23</f>
         <v>10.1105370782339</v>
       </c>
-      <c r="C7" s="14" t="n">
+      <c r="C7" s="18" t="n">
         <f aca="false">Bomba!C30</f>
         <v>0</v>
       </c>
@@ -2635,13 +2822,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>163</v>
-      </c>
-      <c r="B8" s="29" t="n">
+        <v>176</v>
+      </c>
+      <c r="B8" s="28" t="n">
         <f aca="false">Intercambiador!B17</f>
-        <v>224000</v>
-      </c>
-      <c r="C8" s="29" t="n">
+        <v>192000</v>
+      </c>
+      <c r="C8" s="28" t="n">
         <f aca="false">Intercambiador!C24</f>
         <v>0</v>
       </c>
@@ -2652,11 +2839,11 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>164</v>
+        <v>177</v>
       </c>
       <c r="B9" s="32" t="n">
         <f aca="false">Fermentador!B21</f>
-        <v>0.0748617436564737</v>
+        <v>0.074433962264151</v>
       </c>
       <c r="C9" s="32" t="n">
         <f aca="false">Fermentador!B26</f>
@@ -2669,7 +2856,7 @@
     </row>
     <row r="11" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>165</v>
+        <v>178</v>
       </c>
       <c r="B11" s="4"/>
       <c r="C11" s="4"/>

</xml_diff>